<commit_message>
update excel file date
</commit_message>
<xml_diff>
--- a/E5 -Tableau de synthese.xlsx
+++ b/E5 -Tableau de synthese.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BTS\Portfolio_BTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C2E2809-E50E-4567-8D26-D8F867BDBD80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FDBD08B-BCA0-490C-B50C-C8F67F93A4E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="38">
   <si>
     <t>Gérer le patrimoine informatique</t>
   </si>
@@ -128,9 +128,6 @@
     <t>X</t>
   </si>
   <si>
-    <t>16/12/2025 au 15/03/25</t>
-  </si>
-  <si>
     <t>NOM et prénom : BOIN Baptiste</t>
   </si>
   <si>
@@ -144,6 +141,21 @@
   </si>
   <si>
     <t>[ ] SISR</t>
+  </si>
+  <si>
+    <t>16/12/2025 au 15/03/2026</t>
+  </si>
+  <si>
+    <t>10/12/2025 au 15/03/2026</t>
+  </si>
+  <si>
+    <t>11/08/2025 au 19/02/2026</t>
+  </si>
+  <si>
+    <t>08/04/2025 au 16/06/2025</t>
+  </si>
+  <si>
+    <t>10/09/2024 au 08/10/2024</t>
   </si>
 </sst>
 </file>
@@ -695,9 +707,48 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -720,45 +771,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1080,83 +1092,83 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25" t="s">
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="H1" s="25"/>
+      <c r="H1" s="27"/>
     </row>
     <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
     </row>
     <row r="3" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="26" t="s">
-        <v>29</v>
-      </c>
-      <c r="B3" s="27"/>
-      <c r="C3" s="27"/>
-      <c r="D3" s="27"/>
-      <c r="E3" s="28"/>
-      <c r="F3" s="32" t="s">
+      <c r="A3" s="39" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" s="40"/>
+      <c r="C3" s="40"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="45" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="27"/>
-      <c r="H3" s="33"/>
+      <c r="G3" s="40"/>
+      <c r="H3" s="46"/>
       <c r="K3" s="9"/>
       <c r="L3" s="9"/>
       <c r="M3" s="9"/>
     </row>
     <row r="4" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="29" t="s">
-        <v>30</v>
-      </c>
-      <c r="B4" s="30"/>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="31"/>
+      <c r="A4" s="42" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="43"/>
+      <c r="C4" s="43"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="44"/>
       <c r="F4" s="10" t="s">
         <v>8</v>
       </c>
       <c r="G4" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:43" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="44" t="s">
-        <v>31</v>
-      </c>
-      <c r="B5" s="45"/>
-      <c r="C5" s="45"/>
-      <c r="D5" s="45"/>
-      <c r="E5" s="45"/>
-      <c r="F5" s="45"/>
-      <c r="G5" s="45"/>
-      <c r="H5" s="46"/>
+      <c r="A5" s="36" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="37"/>
+      <c r="C5" s="37"/>
+      <c r="D5" s="37"/>
+      <c r="E5" s="37"/>
+      <c r="F5" s="37"/>
+      <c r="G5" s="37"/>
+      <c r="H5" s="38"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="34" t="s">
+      <c r="A6" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="42" t="s">
+      <c r="B6" s="34" t="s">
         <v>18</v>
       </c>
       <c r="C6" s="2" t="s">
@@ -1179,8 +1191,8 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="13" customFormat="1" ht="324.89999999999998" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="35"/>
-      <c r="B7" s="43"/>
+      <c r="A7" s="26"/>
+      <c r="B7" s="35"/>
       <c r="C7" s="4" t="s">
         <v>9</v>
       </c>
@@ -1236,16 +1248,16 @@
       <c r="AQ7" s="8"/>
     </row>
     <row r="8" spans="1:43" s="13" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A8" s="36" t="s">
+      <c r="A8" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="37"/>
-      <c r="C8" s="37"/>
-      <c r="D8" s="37"/>
-      <c r="E8" s="37"/>
-      <c r="F8" s="37"/>
-      <c r="G8" s="37"/>
-      <c r="H8" s="38"/>
+      <c r="B8" s="29"/>
+      <c r="C8" s="29"/>
+      <c r="D8" s="29"/>
+      <c r="E8" s="29"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="29"/>
+      <c r="H8" s="30"/>
       <c r="I8" s="8"/>
       <c r="J8" s="8"/>
       <c r="K8" s="8"/>
@@ -1286,7 +1298,9 @@
       <c r="A9" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="14"/>
+      <c r="B9" s="14" t="s">
+        <v>35</v>
+      </c>
       <c r="C9" s="15"/>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
@@ -1335,7 +1349,9 @@
       <c r="A10" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="14"/>
+      <c r="B10" s="14" t="s">
+        <v>34</v>
+      </c>
       <c r="C10" s="24" t="s">
         <v>27</v>
       </c>
@@ -1430,16 +1446,16 @@
       <c r="AQ11" s="8"/>
     </row>
     <row r="12" spans="1:43" s="13" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A12" s="39" t="s">
+      <c r="A12" s="31" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="40"/>
-      <c r="C12" s="40"/>
-      <c r="D12" s="40"/>
-      <c r="E12" s="40"/>
-      <c r="F12" s="40"/>
-      <c r="G12" s="40"/>
-      <c r="H12" s="41"/>
+      <c r="B12" s="32"/>
+      <c r="C12" s="32"/>
+      <c r="D12" s="32"/>
+      <c r="E12" s="32"/>
+      <c r="F12" s="32"/>
+      <c r="G12" s="32"/>
+      <c r="H12" s="33"/>
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
       <c r="K12" s="8"/>
@@ -1480,7 +1496,9 @@
       <c r="A13" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="14"/>
+      <c r="B13" s="14" t="s">
+        <v>36</v>
+      </c>
       <c r="C13" s="24" t="s">
         <v>27</v>
       </c>
@@ -1531,7 +1549,9 @@
       <c r="A14" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="14"/>
+      <c r="B14" s="14" t="s">
+        <v>37</v>
+      </c>
       <c r="C14" s="24" t="s">
         <v>27</v>
       </c>
@@ -1626,16 +1646,16 @@
       <c r="AQ15" s="8"/>
     </row>
     <row r="16" spans="1:43" s="13" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A16" s="39" t="s">
+      <c r="A16" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="40"/>
-      <c r="C16" s="40"/>
-      <c r="D16" s="40"/>
-      <c r="E16" s="40"/>
-      <c r="F16" s="40"/>
-      <c r="G16" s="40"/>
-      <c r="H16" s="41"/>
+      <c r="B16" s="32"/>
+      <c r="C16" s="32"/>
+      <c r="D16" s="32"/>
+      <c r="E16" s="32"/>
+      <c r="F16" s="32"/>
+      <c r="G16" s="32"/>
+      <c r="H16" s="33"/>
       <c r="I16" s="8"/>
       <c r="J16" s="8"/>
       <c r="K16" s="8"/>
@@ -1677,7 +1697,7 @@
         <v>26</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="C17" s="24" t="s">
         <v>27</v>
@@ -1867,6 +1887,11 @@
     <row r="65" s="8" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
@@ -1874,11 +1899,6 @@
     <mergeCell ref="A16:H16"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>